<commit_message>
feat: Implement Next-Gen Multi-Agent Architecture and Data Intelligence Engine
- Settings-based plugin registry in config/regions/ and dynamic loader scripts/core/region_manager.py
- Data Intelligence Agent in scripts/data_intelligence_engine.py with 1:1 lineup gaps, WoW trends, and executive briefing report
- AI Executive Summary tab integrated into eu_price_dashboard_template.html and generate_eu_dashboard.py
- Master Orchestrator CLI in scripts/orchestrator.py and subagent spec in .agents/subagents/data_intelligence_agent.md
- Updated project rules in AGENTS.md, swiss_tv_tracker skill, and tv-price-tracker skill
</commit_message>
<xml_diff>
--- a/data/Swiss_ATA_Comparison_2026_0912.xlsx
+++ b/data/Swiss_ATA_Comparison_2026_0912.xlsx
@@ -2575,21 +2575,13 @@
       <c r="J27" s="89" t="inlineStr"/>
       <c r="K27" s="89" t="inlineStr"/>
       <c r="L27" s="90" t="inlineStr"/>
-      <c r="M27" s="125" t="inlineStr">
-        <is>
-          <t>QE83S90FAE</t>
-        </is>
-      </c>
+      <c r="M27" s="125" t="inlineStr"/>
       <c r="N27" s="89">
         <f>IF(O27="","",O27-P27)</f>
         <v/>
       </c>
-      <c r="O27" s="89" t="n">
-        <v>3899</v>
-      </c>
-      <c r="P27" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O27" s="89" t="inlineStr"/>
+      <c r="P27" s="89" t="inlineStr"/>
       <c r="Q27" s="90" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1" s="55">
@@ -3686,21 +3678,13 @@
         <f>IFERROR(I50/I7,"")</f>
         <v/>
       </c>
-      <c r="M50" s="83" t="inlineStr">
-        <is>
-          <t>55QNED80A6A</t>
-        </is>
-      </c>
+      <c r="M50" s="83" t="inlineStr"/>
       <c r="N50" s="84">
         <f>IF(O50="","",O50-P50)</f>
         <v/>
       </c>
-      <c r="O50" s="84" t="n">
-        <v>701</v>
-      </c>
-      <c r="P50" s="84" t="n">
-        <v>0</v>
-      </c>
+      <c r="O50" s="84" t="inlineStr"/>
+      <c r="P50" s="84" t="inlineStr"/>
       <c r="Q50" s="85">
         <f>IFERROR(N50/N7,"")</f>
         <v/>
@@ -3994,21 +3978,13 @@
       <c r="J56" s="96" t="inlineStr"/>
       <c r="K56" s="96" t="inlineStr"/>
       <c r="L56" s="90" t="inlineStr"/>
-      <c r="M56" s="125" t="inlineStr">
-        <is>
-          <t>QE65QN80FAU</t>
-        </is>
-      </c>
+      <c r="M56" s="125" t="inlineStr"/>
       <c r="N56" s="95">
         <f>IF(O56="","",O56-P56)</f>
         <v/>
       </c>
-      <c r="O56" s="89" t="n">
-        <v>1559</v>
-      </c>
-      <c r="P56" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O56" s="89" t="inlineStr"/>
+      <c r="P56" s="89" t="inlineStr"/>
       <c r="Q56" s="90" t="inlineStr"/>
     </row>
     <row r="57" ht="20" customHeight="1" s="55">
@@ -4054,21 +4030,13 @@
         <v>0</v>
       </c>
       <c r="L57" s="90" t="inlineStr"/>
-      <c r="M57" s="125" t="inlineStr">
-        <is>
-          <t>QE55QN80FAU</t>
-        </is>
-      </c>
+      <c r="M57" s="125" t="inlineStr"/>
       <c r="N57" s="95">
         <f>IF(O57="","",O57-P57)</f>
         <v/>
       </c>
-      <c r="O57" s="96" t="n">
-        <v>1325</v>
-      </c>
-      <c r="P57" s="96" t="n">
-        <v>0</v>
-      </c>
+      <c r="O57" s="96" t="inlineStr"/>
+      <c r="P57" s="96" t="inlineStr"/>
       <c r="Q57" s="90" t="inlineStr"/>
     </row>
     <row r="58" ht="20" customHeight="1" s="55">
@@ -4289,21 +4257,13 @@
         <v>0</v>
       </c>
       <c r="L62" s="90" t="inlineStr"/>
-      <c r="M62" s="125" t="inlineStr">
-        <is>
-          <t>QE65QN70FAU</t>
-        </is>
-      </c>
+      <c r="M62" s="125" t="inlineStr"/>
       <c r="N62" s="89">
         <f>IF(O62="","",O62-P62)</f>
         <v/>
       </c>
-      <c r="O62" s="89" t="n">
-        <v>943</v>
-      </c>
-      <c r="P62" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O62" s="89" t="inlineStr"/>
+      <c r="P62" s="89" t="inlineStr"/>
       <c r="Q62" s="90" t="inlineStr"/>
     </row>
     <row r="63" ht="20" customHeight="1" s="55">
@@ -4341,21 +4301,13 @@
         <v>0</v>
       </c>
       <c r="L63" s="90" t="inlineStr"/>
-      <c r="M63" s="125" t="inlineStr">
-        <is>
-          <t>QE55QN70FAU</t>
-        </is>
-      </c>
+      <c r="M63" s="125" t="inlineStr"/>
       <c r="N63" s="89">
         <f>IF(O63="","",O63-P63)</f>
         <v/>
       </c>
-      <c r="O63" s="89" t="n">
-        <v>812</v>
-      </c>
-      <c r="P63" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O63" s="89" t="inlineStr"/>
+      <c r="P63" s="89" t="inlineStr"/>
       <c r="Q63" s="90" t="inlineStr"/>
     </row>
     <row r="64">
@@ -4797,7 +4749,7 @@
       <c r="L73" s="90" t="inlineStr"/>
       <c r="M73" s="125" t="inlineStr">
         <is>
-          <t>QE75Q7F5AU</t>
+          <t>QE75Q7FAAU</t>
         </is>
       </c>
       <c r="N73" s="89">
@@ -4805,7 +4757,7 @@
         <v/>
       </c>
       <c r="O73" s="89" t="n">
-        <v>1637</v>
+        <v>1059</v>
       </c>
       <c r="P73" s="89" t="n">
         <v>0</v>
@@ -4935,21 +4887,13 @@
         <v>0</v>
       </c>
       <c r="L76" s="90" t="inlineStr"/>
-      <c r="M76" s="125" t="inlineStr">
-        <is>
-          <t>QE50Q7FAAU</t>
-        </is>
-      </c>
+      <c r="M76" s="125" t="inlineStr"/>
       <c r="N76" s="89">
         <f>IF(O76="","",O76-P76)</f>
         <v/>
       </c>
-      <c r="O76" s="89" t="n">
-        <v>779</v>
-      </c>
-      <c r="P76" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O76" s="89" t="inlineStr"/>
+      <c r="P76" s="89" t="inlineStr"/>
       <c r="Q76" s="90" t="inlineStr"/>
     </row>
     <row r="77" ht="20" customHeight="1" s="55">
@@ -4979,21 +4923,13 @@
       <c r="J77" s="89" t="inlineStr"/>
       <c r="K77" s="89" t="inlineStr"/>
       <c r="L77" s="90" t="inlineStr"/>
-      <c r="M77" s="125" t="inlineStr">
-        <is>
-          <t>QE43Q7FAAU</t>
-        </is>
-      </c>
+      <c r="M77" s="125" t="inlineStr"/>
       <c r="N77" s="89">
         <f>IF(O77="","",O77-P77)</f>
         <v/>
       </c>
-      <c r="O77" s="89" t="n">
-        <v>609</v>
-      </c>
-      <c r="P77" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O77" s="89" t="inlineStr"/>
+      <c r="P77" s="89" t="inlineStr"/>
       <c r="Q77" s="90" t="inlineStr"/>
     </row>
     <row r="78">
@@ -5048,21 +4984,13 @@
         <f>IFERROR(I79/I4,"")</f>
         <v/>
       </c>
-      <c r="M79" s="83" t="inlineStr">
-        <is>
-          <t>86UA75006LA</t>
-        </is>
-      </c>
+      <c r="M79" s="83" t="inlineStr"/>
       <c r="N79" s="84">
         <f>IF(O79="","",O79-P79)</f>
         <v/>
       </c>
-      <c r="O79" s="84" t="n">
-        <v>1403</v>
-      </c>
-      <c r="P79" s="84" t="n">
-        <v>0</v>
-      </c>
+      <c r="O79" s="84" t="inlineStr"/>
+      <c r="P79" s="84" t="inlineStr"/>
       <c r="Q79" s="85">
         <f>IFERROR(N79/N4,"")</f>
         <v/>
@@ -5154,21 +5082,13 @@
         <f>IFERROR(I81/I6,"")</f>
         <v/>
       </c>
-      <c r="M81" s="83" t="inlineStr">
-        <is>
-          <t>65UA75006LA</t>
-        </is>
-      </c>
+      <c r="M81" s="83" t="inlineStr"/>
       <c r="N81" s="84">
         <f>IF(O81="","",O81-P81)</f>
         <v/>
       </c>
-      <c r="O81" s="84" t="n">
-        <v>662</v>
-      </c>
-      <c r="P81" s="84" t="n">
-        <v>0</v>
-      </c>
+      <c r="O81" s="84" t="inlineStr"/>
+      <c r="P81" s="84" t="inlineStr"/>
       <c r="Q81" s="85">
         <f>IFERROR(N81/N6,"")</f>
         <v/>
@@ -5268,21 +5188,13 @@
         <f>IFERROR(I83/I7,"")</f>
         <v/>
       </c>
-      <c r="M83" s="83" t="inlineStr">
-        <is>
-          <t>50UA75006LA</t>
-        </is>
-      </c>
+      <c r="M83" s="83" t="inlineStr"/>
       <c r="N83" s="84">
         <f>IF(O83="","",O83-P83)</f>
         <v/>
       </c>
-      <c r="O83" s="84" t="n">
-        <v>492</v>
-      </c>
-      <c r="P83" s="84" t="n">
-        <v>0</v>
-      </c>
+      <c r="O83" s="84" t="inlineStr"/>
+      <c r="P83" s="84" t="inlineStr"/>
       <c r="Q83" s="85">
         <f>IFERROR(N83/N7,"")</f>
         <v/>
@@ -5447,21 +5359,13 @@
         <v>0</v>
       </c>
       <c r="L87" s="90" t="inlineStr"/>
-      <c r="M87" s="125" t="inlineStr">
-        <is>
-          <t>UE75U8000F</t>
-        </is>
-      </c>
+      <c r="M87" s="125" t="inlineStr"/>
       <c r="N87" s="89">
         <f>IF(O87="","",O87-P87)</f>
         <v/>
       </c>
-      <c r="O87" s="89" t="n">
-        <v>1048</v>
-      </c>
-      <c r="P87" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O87" s="89" t="inlineStr"/>
+      <c r="P87" s="89" t="inlineStr"/>
       <c r="Q87" s="90" t="inlineStr"/>
     </row>
     <row r="88" ht="20" customHeight="1" s="55">
@@ -8880,7 +8784,7 @@
       </c>
       <c r="M10" s="83" t="inlineStr">
         <is>
-          <t>OLED77C67LA</t>
+          <t>OLED77C6ELB</t>
         </is>
       </c>
       <c r="N10" s="84">
@@ -8888,7 +8792,7 @@
         <v/>
       </c>
       <c r="O10" s="84" t="n">
-        <v>3058</v>
+        <v>2499</v>
       </c>
       <c r="P10" s="84" t="n">
         <v>0</v>
@@ -9018,7 +8922,7 @@
       </c>
       <c r="M12" s="83" t="inlineStr">
         <is>
-          <t>OLED55C67LA</t>
+          <t>OLED55C6ELB</t>
         </is>
       </c>
       <c r="N12" s="84">
@@ -9026,7 +8930,7 @@
         <v/>
       </c>
       <c r="O12" s="84" t="n">
-        <v>1838</v>
+        <v>1599</v>
       </c>
       <c r="P12" s="84" t="n">
         <v>0</v>
@@ -9087,7 +8991,7 @@
       </c>
       <c r="M13" s="83" t="inlineStr">
         <is>
-          <t>OLED48C67LA</t>
+          <t>OLED48C6ELB</t>
         </is>
       </c>
       <c r="N13" s="84">
@@ -9095,7 +8999,7 @@
         <v/>
       </c>
       <c r="O13" s="84" t="n">
-        <v>1716</v>
+        <v>1399</v>
       </c>
       <c r="P13" s="84" t="n">
         <v>0</v>
@@ -9528,21 +9432,13 @@
       <c r="J22" s="89" t="inlineStr"/>
       <c r="K22" s="89" t="inlineStr"/>
       <c r="L22" s="90" t="inlineStr"/>
-      <c r="M22" s="125" t="inlineStr">
-        <is>
-          <t>QE83S99HAEXZU</t>
-        </is>
-      </c>
+      <c r="M22" s="125" t="inlineStr"/>
       <c r="N22" s="89">
         <f>IF(O22="","",O22-P22)</f>
         <v/>
       </c>
-      <c r="O22" s="89" t="n">
-        <v>6718</v>
-      </c>
-      <c r="P22" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O22" s="89" t="inlineStr"/>
+      <c r="P22" s="89" t="inlineStr"/>
       <c r="Q22" s="90" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1" s="55">
@@ -9903,21 +9799,13 @@
       <c r="J30" s="89" t="inlineStr"/>
       <c r="K30" s="89" t="inlineStr"/>
       <c r="L30" s="90" t="inlineStr"/>
-      <c r="M30" s="125" t="inlineStr">
-        <is>
-          <t>QE55S95HFTXZU</t>
-        </is>
-      </c>
+      <c r="M30" s="125" t="inlineStr"/>
       <c r="N30" s="95">
         <f>IF(O30="","",O30-P30)</f>
         <v/>
       </c>
-      <c r="O30" s="96" t="n">
-        <v>3058</v>
-      </c>
-      <c r="P30" s="96" t="n">
-        <v>0</v>
-      </c>
+      <c r="O30" s="96" t="inlineStr"/>
+      <c r="P30" s="96" t="inlineStr"/>
       <c r="Q30" s="90" t="inlineStr"/>
     </row>
     <row r="31" ht="19.9" customHeight="1" s="55">
@@ -10405,21 +10293,13 @@
         <v>0</v>
       </c>
       <c r="L40" s="90" t="inlineStr"/>
-      <c r="M40" s="125" t="inlineStr">
-        <is>
-          <t>QE77S85HAEXZU</t>
-        </is>
-      </c>
+      <c r="M40" s="125" t="inlineStr"/>
       <c r="N40" s="89">
         <f>IF(O40="","",O40-P40)</f>
         <v/>
       </c>
-      <c r="O40" s="89" t="n">
-        <v>3669</v>
-      </c>
-      <c r="P40" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O40" s="89" t="inlineStr"/>
+      <c r="P40" s="89" t="inlineStr"/>
       <c r="Q40" s="90" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1" s="55">
@@ -11031,21 +10911,13 @@
         <f>IFERROR(I52/I7,"")</f>
         <v/>
       </c>
-      <c r="M52" s="88" t="inlineStr">
-        <is>
-          <t>50MRGB87B9B</t>
-        </is>
-      </c>
+      <c r="M52" s="88" t="inlineStr"/>
       <c r="N52" s="89">
         <f>IF(O52="","",O52-P52)</f>
         <v/>
       </c>
-      <c r="O52" s="89" t="n">
-        <v>1350</v>
-      </c>
-      <c r="P52" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O52" s="89" t="inlineStr"/>
+      <c r="P52" s="89" t="inlineStr"/>
       <c r="Q52" s="90">
         <f>IFERROR(N52/N7,"")</f>
         <v/>
@@ -11623,21 +11495,13 @@
         <f>IFERROR(I64/I7,"")</f>
         <v/>
       </c>
-      <c r="M64" s="83" t="inlineStr">
-        <is>
-          <t>43QNED86B6B</t>
-        </is>
-      </c>
+      <c r="M64" s="83" t="inlineStr"/>
       <c r="N64" s="84">
         <f>IF(O64="","",O64-P64)</f>
         <v/>
       </c>
-      <c r="O64" s="84" t="n">
-        <v>862</v>
-      </c>
-      <c r="P64" s="84" t="n">
-        <v>0</v>
-      </c>
+      <c r="O64" s="84" t="inlineStr"/>
+      <c r="P64" s="84" t="inlineStr"/>
       <c r="Q64" s="85">
         <f>IFERROR(N64/N7,"")</f>
         <v/>
@@ -12443,21 +12307,13 @@
       <c r="J80" s="89" t="inlineStr"/>
       <c r="K80" s="89" t="inlineStr"/>
       <c r="L80" s="90" t="inlineStr"/>
-      <c r="M80" s="125" t="inlineStr">
-        <is>
-          <t>MRE85R95HATXZU</t>
-        </is>
-      </c>
+      <c r="M80" s="125" t="inlineStr"/>
       <c r="N80" s="89">
         <f>IF(O80="","",O80-P80)</f>
         <v/>
       </c>
-      <c r="O80" s="89" t="n">
-        <v>6718</v>
-      </c>
-      <c r="P80" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O80" s="89" t="inlineStr"/>
+      <c r="P80" s="89" t="inlineStr"/>
       <c r="Q80" s="90" t="inlineStr"/>
     </row>
     <row r="81" ht="20" customHeight="1" s="55">
@@ -12495,21 +12351,13 @@
         <v>500</v>
       </c>
       <c r="L81" s="90" t="inlineStr"/>
-      <c r="M81" s="125" t="inlineStr">
-        <is>
-          <t>MRE75R95HATXZU</t>
-        </is>
-      </c>
+      <c r="M81" s="125" t="inlineStr"/>
       <c r="N81" s="89">
         <f>IF(O81="","",O81-P81)</f>
         <v/>
       </c>
-      <c r="O81" s="89" t="n">
-        <v>5498</v>
-      </c>
-      <c r="P81" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O81" s="89" t="inlineStr"/>
+      <c r="P81" s="89" t="inlineStr"/>
       <c r="Q81" s="90" t="inlineStr"/>
     </row>
     <row r="82" ht="20" customHeight="1" s="55">
@@ -12539,21 +12387,13 @@
       <c r="J82" s="89" t="inlineStr"/>
       <c r="K82" s="89" t="inlineStr"/>
       <c r="L82" s="90" t="inlineStr"/>
-      <c r="M82" s="125" t="inlineStr">
-        <is>
-          <t>MRE65R95HATXZU</t>
-        </is>
-      </c>
+      <c r="M82" s="125" t="inlineStr"/>
       <c r="N82" s="95">
         <f>IF(O82="","",O82-P82)</f>
         <v/>
       </c>
-      <c r="O82" s="89" t="n">
-        <v>4278</v>
-      </c>
-      <c r="P82" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O82" s="89" t="inlineStr"/>
+      <c r="P82" s="89" t="inlineStr"/>
       <c r="Q82" s="90" t="inlineStr"/>
     </row>
     <row r="83" ht="20" customHeight="1" s="55">
@@ -13009,21 +12849,13 @@
         <v>0</v>
       </c>
       <c r="L92" s="90" t="inlineStr"/>
-      <c r="M92" s="125" t="inlineStr">
-        <is>
-          <t>QE85QN80HAUXXN</t>
-        </is>
-      </c>
+      <c r="M92" s="125" t="inlineStr"/>
       <c r="N92" s="89">
         <f>IF(O92="","",O92-P92)</f>
         <v/>
       </c>
-      <c r="O92" s="89" t="n">
-        <v>2448</v>
-      </c>
-      <c r="P92" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O92" s="89" t="inlineStr"/>
+      <c r="P92" s="89" t="inlineStr"/>
       <c r="Q92" s="90" t="inlineStr"/>
     </row>
     <row r="93" ht="20" customHeight="1" s="55">
@@ -13069,21 +12901,13 @@
         <v>0</v>
       </c>
       <c r="L93" s="90" t="inlineStr"/>
-      <c r="M93" s="125" t="inlineStr">
-        <is>
-          <t>QE75QN80HAUXXN</t>
-        </is>
-      </c>
+      <c r="M93" s="125" t="inlineStr"/>
       <c r="N93" s="89">
         <f>IF(O93="","",O93-P93)</f>
         <v/>
       </c>
-      <c r="O93" s="89" t="n">
-        <v>2815</v>
-      </c>
-      <c r="P93" s="89" t="n">
-        <v>0</v>
-      </c>
+      <c r="O93" s="89" t="inlineStr"/>
+      <c r="P93" s="89" t="inlineStr"/>
       <c r="Q93" s="90" t="inlineStr"/>
     </row>
     <row r="94" ht="20" customHeight="1" s="55">
@@ -14552,7 +14376,7 @@
       <c r="L127" s="90" t="inlineStr"/>
       <c r="M127" s="125" t="inlineStr">
         <is>
-          <t>UE75U8070HUXXN</t>
+          <t>UE75U8090HUXXN</t>
         </is>
       </c>
       <c r="N127" s="96">
@@ -14560,7 +14384,7 @@
         <v/>
       </c>
       <c r="O127" s="89" t="n">
-        <v>1472</v>
+        <v>825</v>
       </c>
       <c r="P127" s="89" t="n">
         <v>0</v>
@@ -14604,7 +14428,7 @@
       <c r="L128" s="90" t="inlineStr"/>
       <c r="M128" s="125" t="inlineStr">
         <is>
-          <t>UE65U8070H</t>
+          <t>UE65U8090HUXXN</t>
         </is>
       </c>
       <c r="N128" s="96">
@@ -14612,7 +14436,7 @@
         <v/>
       </c>
       <c r="O128" s="89" t="n">
-        <v>1106</v>
+        <v>700</v>
       </c>
       <c r="P128" s="89" t="n">
         <v>0</v>
@@ -14656,7 +14480,7 @@
       <c r="L129" s="90" t="inlineStr"/>
       <c r="M129" s="125" t="inlineStr">
         <is>
-          <t>UE55U8070H</t>
+          <t>UE55U8090HUXXN</t>
         </is>
       </c>
       <c r="N129" s="96">
@@ -14664,7 +14488,7 @@
         <v/>
       </c>
       <c r="O129" s="89" t="n">
-        <v>862</v>
+        <v>450</v>
       </c>
       <c r="P129" s="89" t="n">
         <v>0</v>

</xml_diff>